<commit_message>
data: add R1 and R4 creel inputs
</commit_message>
<xml_diff>
--- a/input_files/pst/R1_creel/Salmon Angler Days 2022-2025.xlsx
+++ b/input_files/pst/R1_creel/Salmon Angler Days 2022-2025.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateofwa-my.sharepoint.com/personal/jeremy_trump_dfw_wa_gov/Documents/Documents/Data8/2026/Data Request/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateofwa-my.sharepoint.com/personal/michael_gembala_dfw_wa_gov/Documents/Documents/Data/Data 2026/Data request/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="25" documentId="8_{2D740959-B598-4ABE-9600-8D6C45BE9C3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{68DC46B0-7EA1-4CE1-B959-A2F17A1EC134}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7964BCC0-3061-410C-8BF4-C4453B3DCCA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5CEB1A23-573C-4CA7-8E65-1D1A6AE26B05}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="9">
   <si>
     <t>Species</t>
   </si>
@@ -66,9 +66,6 @@
   </si>
   <si>
     <t>Shore Angler Days</t>
-  </si>
-  <si>
-    <t>Mike Check these also  total of shore and boat is 5000 but total was showing 4990.</t>
   </si>
 </sst>
 </file>
@@ -100,7 +97,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -109,18 +106,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -136,43 +127,6 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -245,29 +199,59 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -602,7 +586,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93A9B654-55B5-45E4-BC2F-7674ED42F06A}">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9.42578125" bestFit="1" customWidth="1"/>
@@ -612,138 +596,135 @@
     <col min="6" max="6" width="16.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B3" s="1" t="s">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B3" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="13" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B4" s="4" t="s">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="2">
         <v>2022</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="7">
         <v>1378</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="7">
         <v>2942</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="8">
         <v>4320</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B5" s="7" t="s">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B5" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="14">
         <v>2023</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="15">
         <v>709</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="15">
         <v>1540</v>
       </c>
-      <c r="F5" s="8">
+      <c r="F5" s="9">
         <v>2249</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B6" s="7" t="s">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B6" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="14">
         <v>2024</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="15">
         <v>587</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="15">
         <v>1211</v>
       </c>
-      <c r="F6" s="8">
+      <c r="F6" s="9">
         <v>1798</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B7" s="9" t="s">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B7" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="14">
         <v>2025</v>
       </c>
-      <c r="D7" s="10">
+      <c r="D7" s="15">
         <v>949</v>
       </c>
-      <c r="E7" s="10">
+      <c r="E7" s="15">
         <v>2172</v>
       </c>
-      <c r="F7" s="11">
+      <c r="F7" s="9">
         <v>3121</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B8" s="4" t="s">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B8" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C8" s="14">
         <v>2022</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="F8" s="9" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B9" s="7" t="s">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B9" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="14">
         <v>2023</v>
       </c>
       <c r="D9" s="16">
-        <v>4827</v>
+        <v>4794</v>
       </c>
       <c r="E9" s="16">
-        <v>173</v>
-      </c>
-      <c r="F9" s="17">
-        <v>4990</v>
-      </c>
-      <c r="G9" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B10" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="F9" s="10">
+        <v>4957</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B10" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="14">
         <v>2024</v>
       </c>
       <c r="D10" s="15">
@@ -752,20 +733,26 @@
       <c r="E10" s="15">
         <v>124</v>
       </c>
-      <c r="F10" s="8">
+      <c r="F10" s="9">
         <v>6456</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B11" s="9" t="s">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B11" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C11" s="10">
+      <c r="C11" s="5">
         <v>2025</v>
       </c>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14"/>
-      <c r="F11" s="12"/>
+      <c r="D11" s="11">
+        <v>5023</v>
+      </c>
+      <c r="E11" s="11">
+        <v>87</v>
+      </c>
+      <c r="F11" s="12">
+        <v>5110</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>